<commit_message>
WIP: save current progress
</commit_message>
<xml_diff>
--- a/audit/source_registry.xlsx
+++ b/audit/source_registry.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MameBARBOSAMONTEIRO\projet01\audit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F61C892-B5CF-4174-BD4D-8288A29049ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{218FBCE5-26B6-4CAC-A5C3-7AFBB8939648}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4248" yWindow="-17280" windowWidth="15552" windowHeight="8376" xr2:uid="{35C0E305-D2F3-40AB-AF23-BDE82A5C9E24}"/>
+    <workbookView xWindow="11112" yWindow="-17280" windowWidth="15552" windowHeight="8376" xr2:uid="{35C0E305-D2F3-40AB-AF23-BDE82A5C9E24}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -101,9 +101,6 @@
     <t>Free</t>
   </si>
   <si>
-    <t>Download / Excel Export</t>
-  </si>
-  <si>
     <t>High</t>
   </si>
   <si>
@@ -393,6 +390,9 @@
   </si>
   <si>
     <t>GOUVERNANCE DES SOURCES</t>
+  </si>
+  <si>
+    <t>HTTP Download</t>
   </si>
 </sst>
 </file>
@@ -514,10 +514,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -875,22 +875,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
+      <c r="A1" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
     </row>
     <row r="3" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="4" spans="1:15" ht="17" thickBot="1" x14ac:dyDescent="0.4">
@@ -914,7 +914,7 @@
         <v>0</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>1</v>
@@ -950,7 +950,7 @@
         <v>15</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="44" thickBot="1" x14ac:dyDescent="0.4">
@@ -958,7 +958,7 @@
         <v>16</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>17</v>
@@ -967,476 +967,476 @@
         <v>18</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G9" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="H9" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>46</v>
       </c>
       <c r="I9" s="6">
         <v>46262</v>
       </c>
       <c r="J9" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="K9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="L9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="L9" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="M9" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="N9" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="73" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>24</v>
-      </c>
       <c r="D10" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="8" t="s">
         <v>52</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>53</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I10" s="6">
         <v>46262</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="M10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="L10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="N10" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O10" s="1"/>
     </row>
     <row r="11" spans="1:15" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E11" s="8" t="s">
         <v>56</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>57</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I11" s="6">
         <v>46262</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L11" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="N11" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="M11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N11" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="O11" s="1"/>
     </row>
     <row r="12" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I12" s="6">
         <v>46262</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L12" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="N12" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>71</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G13" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="I13" s="6">
         <v>46268</v>
       </c>
       <c r="J13" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L13" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="M13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="L13" s="2" t="s">
+      <c r="N13" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="E14" s="8" t="s">
         <v>85</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>86</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G14" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="H14" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="I14" s="6">
         <v>46268</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="M14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="L14" s="2" t="s">
+      <c r="N14" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N14" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I15" s="6">
         <v>46268</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="M15" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="L15" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="N15" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="C16" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="E16" s="8" t="s">
         <v>96</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>97</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I16" s="6">
         <v>46268</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="K16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="M16" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="L16" s="2" t="s">
+      <c r="N16" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N16" s="2" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D17" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="E17" s="8" t="s">
         <v>101</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>102</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I17" s="6">
         <v>46268</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M17" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="L17" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="M17" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="N17" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="58" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C18" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="D18" s="3" t="s">
-        <v>106</v>
-      </c>
       <c r="E18" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G18" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="H18" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="I18" s="6">
         <v>46268</v>
       </c>
       <c r="J18" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="L18" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="K18" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="L18" s="2" t="s">
+      <c r="M18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="N18" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="M18" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N18" s="2" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C19" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>113</v>
-      </c>
       <c r="E19" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I19" s="6">
         <v>46268</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.35">
@@ -1452,14 +1452,14 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="E9" r:id="rId1" xr:uid="{B55F5DAB-0F51-4251-9A62-F393F5C7695C}"/>
-    <hyperlink ref="E10" r:id="rId2" xr:uid="{C6D3FF36-40F5-4A4C-A8B8-994BBA1237A5}"/>
-    <hyperlink ref="E11" r:id="rId3" xr:uid="{B91941BC-466F-475C-AFBF-CEBC6A947578}"/>
-    <hyperlink ref="E12" r:id="rId4" xr:uid="{AA048820-C05F-4DE2-9619-2A5824CF3D1C}"/>
-    <hyperlink ref="E14" r:id="rId5" xr:uid="{CEFDC79D-F6B5-4229-AE19-358C297EDE34}"/>
-    <hyperlink ref="E15" r:id="rId6" xr:uid="{FBD25B48-0766-4E81-B726-C899FBD65F7D}"/>
-    <hyperlink ref="E16" r:id="rId7" xr:uid="{50AEED7E-540F-4BC3-9907-E39A46AF3720}"/>
-    <hyperlink ref="E17" r:id="rId8" xr:uid="{02C16CB4-FCD5-46B9-AFBD-279A2C4C210F}"/>
+    <hyperlink ref="E10" r:id="rId1" xr:uid="{C6D3FF36-40F5-4A4C-A8B8-994BBA1237A5}"/>
+    <hyperlink ref="E11" r:id="rId2" xr:uid="{B91941BC-466F-475C-AFBF-CEBC6A947578}"/>
+    <hyperlink ref="E12" r:id="rId3" xr:uid="{AA048820-C05F-4DE2-9619-2A5824CF3D1C}"/>
+    <hyperlink ref="E14" r:id="rId4" xr:uid="{CEFDC79D-F6B5-4229-AE19-358C297EDE34}"/>
+    <hyperlink ref="E15" r:id="rId5" xr:uid="{FBD25B48-0766-4E81-B726-C899FBD65F7D}"/>
+    <hyperlink ref="E16" r:id="rId6" xr:uid="{50AEED7E-540F-4BC3-9907-E39A46AF3720}"/>
+    <hyperlink ref="E17" r:id="rId7" xr:uid="{02C16CB4-FCD5-46B9-AFBD-279A2C4C210F}"/>
+    <hyperlink ref="E9" r:id="rId8" xr:uid="{B55F5DAB-0F51-4251-9A62-F393F5C7695C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>